<commit_message>
UPDATE : Menambahkan rumus logika IF di dalam file latihan-excel-byGPT-01.xlsx pada folder latihan-excel-dasar-byGPT
</commit_message>
<xml_diff>
--- a/belajar-excel-dasar/latihan-excel-dasar-byGPT/latihan-excel-byGPT-01.xlsx
+++ b/belajar-excel-dasar/latihan-excel-dasar-byGPT/latihan-excel-byGPT-01.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eca2b7f21e501f1c/ドキュメント/belajar-excel-dasar/latihan-excel-byGPT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leonovo\OneDrive\ドキュメント\belajar-excel\belajar-excel-dasar\latihan-excel-dasar-byGPT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{47D7BBD2-6721-48E0-8DD6-A00ACB911265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D995D03-8DD3-46F8-A707-EA015BC5EE48}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7706ADCC-7E51-41BF-ABA5-3B926B4F6EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A6D3F684-F5D6-405C-BD02-216C6A25668E}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
   <si>
     <t>No</t>
   </si>
@@ -99,6 +99,12 @@
 Jurusan Teknik Informatika
 Universitas Al-Washliyah Labuhanbatu</t>
     </r>
+  </si>
+  <si>
+    <t>Grade</t>
+  </si>
+  <si>
+    <t>Keterangan</t>
   </si>
 </sst>
 </file>
@@ -140,7 +146,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -153,14 +159,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -241,11 +241,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -264,17 +301,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -291,6 +334,66 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>182880</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="184731" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0394A8E0-8A13-EDDA-5E52-B3CCADA8634B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3840480" y="1104900"/>
+          <a:ext cx="184731" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -590,27 +693,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F58453CB-FBF8-4E72-B145-D63C3FED1C60}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" customWidth="1"/>
+    <col min="1" max="1" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -626,18 +735,24 @@
       <c r="E3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
+      <c r="G3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="6">
         <v>19</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -646,18 +761,26 @@
       <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="8">
-        <v>90</v>
+      <c r="F4" s="9">
+        <v>69</v>
+      </c>
+      <c r="G4" s="13" t="str">
+        <f>IF(F4&gt;=90,"A",IF(F4&gt;=80,"B",IF(F4&gt;=70,"C",IF(F4&gt;=60,"D","E"))))</f>
+        <v>D</v>
+      </c>
+      <c r="H4" s="13" t="str">
+        <f>IF(F4&gt;=70,"LULUS","TIDAK LULUS")</f>
+        <v>TIDAK LULUS</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="7">
         <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -666,18 +789,26 @@
       <c r="E5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="10">
         <v>89</v>
       </c>
+      <c r="G5" s="13" t="str">
+        <f t="shared" ref="G5:G9" si="0">IF(F5&gt;=90,"A",IF(F5&gt;=80,"B",IF(F5&gt;=70,"C",IF(F5&gt;=60,"D","E"))))</f>
+        <v>B</v>
+      </c>
+      <c r="H5" s="13" t="str">
+        <f t="shared" ref="H5:H9" si="1">IF(F5&gt;=70,"LULUS","TIDAK LULUS")</f>
+        <v>LULUS</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="7">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="7">
         <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -686,18 +817,26 @@
       <c r="E6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="10">
         <v>94</v>
       </c>
+      <c r="G6" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="H6" s="13" t="str">
+        <f t="shared" si="1"/>
+        <v>LULUS</v>
+      </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="7">
         <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -706,18 +845,26 @@
       <c r="E7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="9">
-        <v>86</v>
+      <c r="F7" s="10">
+        <v>56</v>
+      </c>
+      <c r="G7" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>E</v>
+      </c>
+      <c r="H7" s="13" t="str">
+        <f t="shared" si="1"/>
+        <v>TIDAK LULUS</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="7">
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="7">
         <v>19</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -726,18 +873,26 @@
       <c r="E8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="9">
-        <v>80</v>
+      <c r="F8" s="10">
+        <v>72</v>
+      </c>
+      <c r="G8" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>C</v>
+      </c>
+      <c r="H8" s="13" t="str">
+        <f t="shared" si="1"/>
+        <v>LULUS</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="7">
         <v>19</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -746,12 +901,22 @@
       <c r="E9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="10">
         <v>92</v>
+      </c>
+      <c r="G9" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="H9" s="13" t="str">
+        <f t="shared" si="1"/>
+        <v>LULUS</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>